<commit_message>
I worked on finding exogenous variables for the model while also working to comment on as much as I could.
</commit_message>
<xml_diff>
--- a/Water Disposal History.xlsx
+++ b/Water Disposal History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://etswdmail-my.sharepoint.com/personal/lfrideley_etswd_com/Documents/Documents/SARIMA Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="171" documentId="8_{9F342BE3-2F2B-4A33-86FA-5252C47A49C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0786317-38BA-4F04-AA8F-45FD45D92FC4}"/>
+  <xr:revisionPtr revIDLastSave="176" documentId="8_{9F342BE3-2F2B-4A33-86FA-5252C47A49C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DFE77CB-E600-45AB-86F6-5ED5AF928D2C}"/>
   <bookViews>
     <workbookView xWindow="32175" yWindow="1530" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{85408E0C-C59E-4CA0-92DA-6AA07159AB49}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>Month/ Year</t>
   </si>
@@ -136,6 +136,9 @@
   </si>
   <si>
     <t>Total Water Volume 1</t>
+  </si>
+  <si>
+    <t>6-month moving average</t>
   </si>
 </sst>
 </file>
@@ -48315,14 +48318,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62516834-FDAB-45A0-893B-2B6358A8E52F}">
-  <dimension ref="A1:D428"/>
+  <dimension ref="A1:G428"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="27.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>28</v>
       </c>
@@ -48335,8 +48338,11 @@
       <c r="D1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>35796</v>
       </c>
@@ -48344,23 +48350,23 @@
         <v>33775964</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>35827</v>
       </c>
       <c r="B3" s="4">
-        <v>30600608</v>
+        <v>33721886</v>
       </c>
       <c r="C3" s="29">
         <f>B3-B2</f>
-        <v>-3175356</v>
+        <v>-54078</v>
       </c>
       <c r="D3">
         <f>(B2+B4)/2</f>
         <v>33721885.5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>35855</v>
       </c>
@@ -48369,14 +48375,14 @@
       </c>
       <c r="C4" s="29">
         <f t="shared" ref="C4:C67" si="0">B4-B3</f>
-        <v>3067199</v>
+        <v>-54079</v>
       </c>
       <c r="D4">
         <f t="shared" ref="D4:D67" si="1">(B3+B5)/2</f>
-        <v>31181405</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>32742044</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>35886</v>
       </c>
@@ -48392,7 +48398,7 @@
         <v>33083817.5</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>35916</v>
       </c>
@@ -48408,7 +48414,7 @@
         <v>31276953.5</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>35947</v>
       </c>
@@ -48424,7 +48430,7 @@
         <v>31833535.5</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>35977</v>
       </c>
@@ -48440,7 +48446,7 @@
         <v>30624828</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>36008</v>
       </c>
@@ -48456,7 +48462,7 @@
         <v>30066511.5</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>36039</v>
       </c>
@@ -48472,7 +48478,7 @@
         <v>30209072.5</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>36069</v>
       </c>
@@ -48488,7 +48494,7 @@
         <v>28534857.5</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>36100</v>
       </c>
@@ -48504,7 +48510,7 @@
         <v>28897874.5</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>36130</v>
       </c>
@@ -48520,7 +48526,7 @@
         <v>27652255.5</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>36161</v>
       </c>
@@ -48536,7 +48542,7 @@
         <v>27440151.5</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>36192</v>
       </c>
@@ -48552,7 +48558,7 @@
         <v>27044747.5</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>36220</v>
       </c>
@@ -49797,7 +49803,7 @@
       </c>
       <c r="D93">
         <f t="shared" si="3"/>
-        <v>28343494.5</v>
+        <v>29846313.5</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
@@ -49805,11 +49811,11 @@
         <v>38596</v>
       </c>
       <c r="B94" s="8">
-        <v>27032542</v>
+        <v>30038180</v>
       </c>
       <c r="C94" s="29">
         <f t="shared" si="2"/>
-        <v>-3056873</v>
+        <v>-51235</v>
       </c>
       <c r="D94">
         <f t="shared" si="3"/>
@@ -49825,11 +49831,11 @@
       </c>
       <c r="C95" s="29">
         <f t="shared" si="2"/>
-        <v>2954403</v>
+        <v>-51235</v>
       </c>
       <c r="D95">
         <f t="shared" si="3"/>
-        <v>28201748.5</v>
+        <v>29704567.5</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
@@ -51413,7 +51419,7 @@
       </c>
       <c r="D194">
         <f t="shared" si="5"/>
-        <v>32706390</v>
+        <v>33780377.5</v>
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.25">
@@ -51421,11 +51427,11 @@
         <v>41671</v>
       </c>
       <c r="B195" s="8">
-        <v>31221548</v>
+        <v>33369523</v>
       </c>
       <c r="C195" s="29">
         <f t="shared" si="4"/>
-        <v>-2558760</v>
+        <v>-410785</v>
       </c>
       <c r="D195">
         <f t="shared" si="5"/>
@@ -51441,11 +51447,11 @@
       </c>
       <c r="C196" s="29">
         <f t="shared" ref="C196:C259" si="6">B196-B195</f>
-        <v>1737189</v>
+        <v>-410786</v>
       </c>
       <c r="D196">
         <f t="shared" ref="D196:D259" si="7">(B195+B197)/2</f>
-        <v>32305335</v>
+        <v>33379322.5</v>
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.25">
@@ -51637,7 +51643,7 @@
       </c>
       <c r="D208">
         <f t="shared" si="7"/>
-        <v>34187889</v>
+        <v>34911337.5</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
@@ -51645,11 +51651,11 @@
         <v>42095</v>
       </c>
       <c r="B209" s="8">
-        <v>33129257</v>
+        <v>34576154</v>
       </c>
       <c r="C209" s="29">
         <f t="shared" si="6"/>
-        <v>-2276367</v>
+        <v>-829470</v>
       </c>
       <c r="D209">
         <f t="shared" si="7"/>
@@ -51665,11 +51671,11 @@
       </c>
       <c r="C210" s="29">
         <f t="shared" si="6"/>
-        <v>617426</v>
+        <v>-829471</v>
       </c>
       <c r="D210">
         <f t="shared" si="7"/>
-        <v>32877254</v>
+        <v>33600702.5</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
@@ -54102,12 +54108,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="1bd1721e-2220-476a-8a0c-275704810b64">
+      <UserInfo>
+        <DisplayName>Carter Matthews</DisplayName>
+        <AccountId>16</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3d892915-ebce-4bfc-a614-64709b81479e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="1bd1721e-2220-476a-8a0c-275704810b64" xsi:nil="true"/>
+    <AFEDate xmlns="3d892915-ebce-4bfc-a614-64709b81479e" xsi:nil="true"/>
+    <IntacctPROJNo_x002e_ xmlns="3d892915-ebce-4bfc-a614-64709b81479e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -54348,29 +54365,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="1bd1721e-2220-476a-8a0c-275704810b64">
-      <UserInfo>
-        <DisplayName>Carter Matthews</DisplayName>
-        <AccountId>16</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3d892915-ebce-4bfc-a614-64709b81479e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="1bd1721e-2220-476a-8a0c-275704810b64" xsi:nil="true"/>
-    <AFEDate xmlns="3d892915-ebce-4bfc-a614-64709b81479e" xsi:nil="true"/>
-    <IntacctPROJNo_x002e_ xmlns="3d892915-ebce-4bfc-a614-64709b81479e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53071905-3A2E-49BD-A006-8C150C715FC8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA15176D-9C18-4E3E-9223-CD0FCCE499CD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="3d892915-ebce-4bfc-a614-64709b81479e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="1bd1721e-2220-476a-8a0c-275704810b64"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -54395,18 +54410,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA15176D-9C18-4E3E-9223-CD0FCCE499CD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53071905-3A2E-49BD-A006-8C150C715FC8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="3d892915-ebce-4bfc-a614-64709b81479e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="1bd1721e-2220-476a-8a0c-275704810b64"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>